<commit_message>
Refactor timestamp handling and note tagging in ScanWindow for improved clarity and consistency
</commit_message>
<xml_diff>
--- a/Sessions/2nd October session 1.xlsx
+++ b/Sessions/2nd October session 1.xlsx
@@ -512,8 +512,18 @@
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>12:42:30 AM</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>[12:42:30 AM] Attended (Didn't do Exam &amp; Homework).
+[12:43:04 AM] Canceled.
+[12:42:30 AM] Attended (Didn't do Exam &amp; Homework).</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -549,8 +559,16 @@
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>12:42:56 AM</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>[12:43:17 AM] Canceled.</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -594,8 +612,46 @@
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>12:44:06 AM</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>[12:44:06 AM] Completed Exam &amp; Homework at center.
+[12:45:33 AM] Canceled.
+[12:44:06 AM] Completed Exam &amp; Homework at center.
+[12:45:36 AM] Attended (Didn't do Exam &amp; Homework).
+[12:44:06 AM] Completed Exam &amp; Homework at center.
+[12:45:33 AM] Canceled.
+[12:44:06 AM] Completed Exam &amp; Homework at center.
+[12:45:39 AM] Canceled.
+[12:44:06 AM] Completed Exam &amp; Homework at center.
+[12:45:33 AM] Canceled.
+[12:44:06 AM] Completed Exam &amp; Homework at center.
+[12:45:36 AM] Attended (Didn't do Exam &amp; Homework).
+[12:44:06 AM] Completed Exam &amp; Homework at center.
+[12:45:33 AM] Canceled.
+[12:44:06 AM] Completed Exam &amp; Homework at center.
+[12:45:41 AM] Denied Entry: No Exam &amp; Homework.
+[12:44:06 AM] Completed Exam &amp; Homework at center.
+[12:45:33 AM] Canceled.
+[12:44:06 AM] Completed Exam &amp; Homework at center.
+[12:45:36 AM] Attended (Didn't do Exam &amp; Homework).
+[12:44:06 AM] Completed Exam &amp; Homework at center.
+[12:45:33 AM] Canceled.
+[12:44:06 AM] Completed Exam &amp; Homework at center.
+[12:45:39 AM] Canceled.
+[12:44:06 AM] Completed Exam &amp; Homework at center.
+[12:45:33 AM] Canceled.
+[12:44:06 AM] Completed Exam &amp; Homework at center.
+[12:45:36 AM] Attended (Didn't do Exam &amp; Homework).
+[12:44:06 AM] Completed Exam &amp; Homework at center.
+[12:45:33 AM] Canceled.
+[12:44:06 AM] Completed Exam &amp; Homework at center.</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>excel_import</t>

</xml_diff>

<commit_message>
Refactor note collection logic in ScanWindow for improved handling of raw text and cleaning process
</commit_message>
<xml_diff>
--- a/Sessions/2nd October session 1.xlsx
+++ b/Sessions/2nd October session 1.xlsx
@@ -731,9 +731,27 @@
           <t>null 5</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>12:54:12 AM</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>[12:54:12 AM] Attended (Didn't do Exam &amp; Homework).
+[12:55:04 AM] Canceled.
+[12:54:12 AM] Attended (Didn't do Exam &amp; Homework).
+[12:56:06 AM] Completed Exam &amp; Homework at center.
+[12:54:12 AM] Attended (Didn't do Exam &amp; Homework).
+[12:55:04 AM] Canceled.
+[12:54:12 AM] Attended (Didn't do Exam &amp; Homework).</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -1214,9 +1232,23 @@
           <t>null 16</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>01:07:20 AM</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>[01:07:20 AM] Attended (Didn't do Exam &amp; Homework).
+[01:07:24 AM] Canceled.
+[01:07:51 AM] Completed Exam &amp; Homework at center.</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
           <t>excel_import</t>

</xml_diff>

<commit_message>
Update default notes in AddStudentDialog and ScanWindow for consistency
</commit_message>
<xml_diff>
--- a/Sessions/2nd October session 1.xlsx
+++ b/Sessions/2nd October session 1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K97"/>
+  <dimension ref="A1:K99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4689,6 +4689,88 @@
       </c>
       <c r="K97" t="inlineStr"/>
     </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>ghghg</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>jtfysksfykjs</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>frxytyksrryk</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Unknown 1</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>01:12:55 AM</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>[01:12:55 AM] manual addition</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>123456</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>asdfgh</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>123456789</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Unknown 2</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>01:26:19 AM</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>[01:26:19 AM] Manually added</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr"/>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>